<commit_message>
Add Тех долг to the plan type list.
The Excel dropdown now offers деливери, дискавери and Тех долг.

Co-authored-by: bbenicore-web <bbenicore-web@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/templates/calendarization_current_plan.xlsx
+++ b/templates/calendarization_current_plan.xlsx
@@ -690,7 +690,7 @@
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Тип — только деливери или дискавери, либо пусто. ЦКО не пишите.</t>
+          <t>Тип — деливери, дискавери или Тех долг, либо пусто. ЦКО не пишите.</t>
         </is>
       </c>
     </row>
@@ -974,6 +974,11 @@
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>ДГП</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Тех долг</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -21953,7 +21958,7 @@
       <formula1>=Справочник!$A$2:$A$6</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D281" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Неверное значение" error="Выберите значение из списка — так не будет разночтений." type="list">
-      <formula1>=Справочник!$C$2:$C$3</formula1>
+      <formula1>=Справочник!$C$2:$C$4</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E281" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Неверное значение" error="Выберите значение из списка — так не будет разночтений." type="list">
       <formula1>=Справочник!$E$2:$E$38</formula1>

</xml_diff>